<commit_message>
Fix remaining 13 broken translations across XLSX design documents
- Dimensional Gate: unavailable situations, sort order, activation state
- Adventure Journal: reward display, stage 1+ entries
- Season Pass: greyed out states, weekly mission progress
- Map/Minimap: teleport description, area completion image

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/SeasonPass_DesignDocument.xlsx
+++ b/docs/SeasonPass_DesignDocument.xlsx
@@ -2325,7 +2325,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M42"/>
+  <dimension ref="A2:M42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="4.375" customWidth="1" style="27" min="1" max="1"/>
@@ -2337,7 +2337,6 @@
     <col width="9" customWidth="1" style="27" min="17" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2" ht="22" customHeight="1" s="72">
       <c r="B2" s="91" t="inlineStr">
         <is>
@@ -3471,7 +3470,7 @@
       <c r="D118" s="88" t="n"/>
       <c r="E118" s="16" t="inlineStr">
         <is>
-          <t>Greyscale processing And green V Check</t>
+          <t>Greyed out with green checkmark when completed</t>
         </is>
       </c>
     </row>
@@ -3682,7 +3681,7 @@
       <c r="D159" s="86" t="n"/>
       <c r="E159" s="20" t="inlineStr">
         <is>
-          <t>Corresponding List Greyscale processing, Reward Icon green V Display</t>
+          <t>Completed entries greyed out; reward icon shows green checkmark</t>
         </is>
       </c>
     </row>
@@ -3739,7 +3738,7 @@
       <c r="D164" s="87" t="n"/>
       <c r="E164" s="71" t="inlineStr">
         <is>
-          <t>Claim Available Reward without case Greyscale processing</t>
+          <t>Greyed out when no claimable rewards available</t>
         </is>
       </c>
     </row>
@@ -4150,7 +4149,7 @@
     <row r="233" ht="16.5" customFormat="1" customHeight="1" s="9">
       <c r="C233" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve"> when) Below and as follows Composition when, Weekly Mission Progressduring state in Monster 100creatures DefeatDid, season Mission Monster 90/100 to Count Done/Applied</t>
+          <t>When composed as below, Weekly Mission remains in progress state</t>
         </is>
       </c>
     </row>

</xml_diff>